<commit_message>
modified:   data/chapter2/extracts/combined_photo.xlsx 	modified:   notebooks/chapter_02/photosynthetic_pathways.ipynb 	modified:   notebooks/chapter_02/subsetting.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/extracts/combined_photo.xlsx
+++ b/data/chapter2/extracts/combined_photo.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/extracts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{7D050F06-588E-46DF-8FE1-528A474EC6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{29E94FE6-457B-4AD6-88FF-5A285B9E0A29}"/>
+  <xr:revisionPtr revIDLastSave="71" documentId="8_{7D050F06-588E-46DF-8FE1-528A474EC6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A4C3416-8599-4781-984E-F922AE49972B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{431B909E-94A0-4438-ACD9-CFFF2AFE3F3D}"/>
   </bookViews>
@@ -2644,7 +2644,31 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="13">
+  <dxfs count="14">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF00B050"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -2701,11 +2725,11 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{5A45568C-C66D-44A2-A02A-01C486D25F65}" name="fred_p" displayName="fred_p" ref="A1:E639" totalsRowShown="0">
   <autoFilter ref="A1:E639" xr:uid="{5A45568C-C66D-44A2-A02A-01C486D25F65}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{D868288D-5A57-4C2E-9EC5-7A679D7ADF78}" name="binominal" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{3002E450-8742-449C-8CFE-4E8EA1516386}" name="F00004" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{E5E712B5-1638-4A15-A23A-D433B6E81C0B}" name="F01286" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{A38A5E90-7517-4239-B32E-4540E782A851}" name="F01287" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{D575187C-6181-4D9B-9BDE-2A7E12706C2B}" name="F00043" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{D868288D-5A57-4C2E-9EC5-7A679D7ADF78}" name="binominal" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{3002E450-8742-449C-8CFE-4E8EA1516386}" name="F00004" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{E5E712B5-1638-4A15-A23A-D433B6E81C0B}" name="F01286" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{A38A5E90-7517-4239-B32E-4540E782A851}" name="F01287" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{D575187C-6181-4D9B-9BDE-2A7E12706C2B}" name="F00043" dataDxfId="9"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2715,10 +2739,10 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{68BB1CAD-A75D-4CC7-B34A-81758268325B}" name="groot_p" displayName="groot_p" ref="A1:D196" totalsRowShown="0">
   <autoFilter ref="A1:D196" xr:uid="{68BB1CAD-A75D-4CC7-B34A-81758268325B}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{D55C34B9-CDC9-4C08-8B82-E2A899C48B34}" name="binominal" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{9A12FF38-8EF9-4388-B223-1719BEEB5B4C}" name="photosyntheticPathway" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{27340414-6F6E-4FB8-AFF5-0AE22EBB0894}" name="references" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{549A7B36-9DF2-4CF2-986E-4C8E5C6AF233}" name="referencesDataset" dataDxfId="4"/>
+    <tableColumn id="1" xr3:uid="{D55C34B9-CDC9-4C08-8B82-E2A899C48B34}" name="binominal" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{9A12FF38-8EF9-4388-B223-1719BEEB5B4C}" name="photosyntheticPathway" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{27340414-6F6E-4FB8-AFF5-0AE22EBB0894}" name="references" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{549A7B36-9DF2-4CF2-986E-4C8E5C6AF233}" name="referencesDataset" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2728,12 +2752,25 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{0F7DB963-8D8C-4EED-BA92-829FC5E365C4}" name="try_p" displayName="try_p" ref="A1:D831" totalsRowShown="0">
   <autoFilter ref="A1:D831" xr:uid="{0F7DB963-8D8C-4EED-BA92-829FC5E365C4}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{21AD1F30-6401-4B2E-85F4-742BBBE3B2B4}" name="Dataset" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{D765FC8D-999A-4470-8835-8D2D5A67B5FC}" name="SpeciesName" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{2BC2CC0B-0CDB-4964-9CF4-7D98F7E667F5}" name="AccSpeciesName" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{5447D786-3B27-4740-9A0B-AA5C6E847B6D}" name="OrigValueStr" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{21AD1F30-6401-4B2E-85F4-742BBBE3B2B4}" name="Dataset" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{D765FC8D-999A-4470-8835-8D2D5A67B5FC}" name="SpeciesName" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{2BC2CC0B-0CDB-4964-9CF4-7D98F7E667F5}" name="AccSpeciesName" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{5447D786-3B27-4740-9A0B-AA5C6E847B6D}" name="OrigValueStr" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D0711551-CB02-441F-BEAD-E2C7A9C6F4A4}" name="Table5" displayName="Table5" ref="A1:D834" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D834" xr:uid="{D0711551-CB02-441F-BEAD-E2C7A9C6F4A4}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{9D60A2B0-4B4A-4621-A6C3-460693FFAE4D}" name="binominal"/>
+    <tableColumn id="2" xr3:uid="{3D80276D-7F3A-4544-A6BC-27A56A4E6484}" name="pathway"/>
+    <tableColumn id="3" xr3:uid="{D8B2DC0E-16A9-4E2F-AC61-1D47D6A56FFC}" name="reference"/>
+    <tableColumn id="4" xr3:uid="{17F90A6A-06D8-4216-A9EF-44AF571B4360}" name="source"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -51670,9 +51707,12 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.5703125" customWidth="1"/>
     <col min="3" max="3" width="255.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.28515625" customWidth="1"/>
+    <col min="8" max="8" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -63358,6 +63398,9 @@
     <sortCondition ref="D2:D834"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
new file:   data/chapter2/FREDv3subset/FRED_subset_collab_categorical.csv 	modified:   data/chapter2/extracts/combined_myco.xlsx 	modified:   data/chapter2/extracts/combined_photo.xlsx 	modified:   notebooks/chapter_02/mycorrhizal_states.ipynb 	modified:   notebooks/chapter_02/subsetting.ipynb
</commit_message>
<xml_diff>
--- a/data/chapter2/extracts/combined_photo.xlsx
+++ b/data/chapter2/extracts/combined_photo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90963425_westernsydney_edu_au/Documents/PhD/code/data/chapter2/extracts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="71" documentId="8_{7D050F06-588E-46DF-8FE1-528A474EC6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A4C3416-8599-4781-984E-F922AE49972B}"/>
+  <xr:revisionPtr revIDLastSave="72" documentId="8_{7D050F06-588E-46DF-8FE1-528A474EC6EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A3756D03-470E-4757-AB9F-C2C903581382}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{431B909E-94A0-4438-ACD9-CFFF2AFE3F3D}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{431B909E-94A0-4438-ACD9-CFFF2AFE3F3D}"/>
   </bookViews>
   <sheets>
     <sheet name="fred" sheetId="2" r:id="rId1"/>
@@ -3098,7 +3098,7 @@
     <col min="2" max="2" width="255.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="3.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>